<commit_message>
✅ Freeze ejecutado: roster y freeze_time actualizados
</commit_message>
<xml_diff>
--- a/data/processed/daily_rosters_excels/roster_2025-12-07.xlsx
+++ b/data/processed/daily_rosters_excels/roster_2025-12-07.xlsx
@@ -1397,16 +1397,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>5105623</v>
+        <v>4869780</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Kel'el Ware</t>
+          <t>Derik Queen</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>NOP</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1642276</t>
+          <t>1642852</t>
         </is>
       </c>
     </row>
@@ -1435,26 +1435,26 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>4869780</v>
+        <v>4433083</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Derik Queen</t>
+          <t>Cam Spencer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>NOP</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1642852</t>
+          <t>1642285</t>
         </is>
       </c>
     </row>
@@ -1473,26 +1473,26 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4433083</v>
+        <v>3032976</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Cam Spencer</t>
+          <t>Rudy Gobert</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1642285</t>
+          <t>203497</t>
         </is>
       </c>
     </row>
@@ -3069,26 +3069,26 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>3138196</v>
+        <v>4898371</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Cameron Johnson</t>
+          <t>Maxime Raynaud</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>SAC</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1629661</t>
+          <t>1642875</t>
         </is>
       </c>
     </row>
@@ -4133,26 +4133,26 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>2528426</v>
+        <v>4278585</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Jordan Clarkson</t>
+          <t>Collin Gillespie</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>NYK</t>
+          <t>PHO</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>203903</t>
+          <t>1631221</t>
         </is>
       </c>
     </row>
@@ -4551,26 +4551,26 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>3102530</v>
+        <v>4591725</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Jusuf Nurkic</t>
+          <t>Ryan Rollins</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>UTA</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>203994</t>
+          <t>1631157</t>
         </is>
       </c>
     </row>
@@ -4589,26 +4589,26 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>4591725</v>
+        <v>3134908</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Ryan Rollins</t>
+          <t>Jakob Poeltl</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1631157</t>
+          <t>1627751</t>
         </is>
       </c>
     </row>
@@ -4627,26 +4627,26 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>3134908</v>
+        <v>4433629</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Jakob Poeltl</t>
+          <t>Ryan Nembhard</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1627751</t>
+          <t>1642948</t>
         </is>
       </c>
     </row>
@@ -4665,26 +4665,26 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>4433629</v>
+        <v>4065731</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Ryan Nembhard</t>
+          <t>Jay Huff</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1642948</t>
+          <t>1630643</t>
         </is>
       </c>
     </row>

</xml_diff>